<commit_message>
docs(4a-13): close Stripe webhook cutover -- F60 resolved, F75 found+fixed
Session 4A-13 (Phase 4X gate 1/3): dual-delivery Stripe webhook endpoint
proven end-to-end on a real production checkout.session.completed event
after fixing a live money_svc Postgres grant gap (F75) the cutover itself
surfaced. F49 (dLocal) PRE-DRAFTed as 4A-14. No application code changed --
the fix was a database GRANT, Davin-directed and Davin-authorized.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/migration-orders/davin-operational-manual/antigravity/migration-process-handbook-antigravity-v12.xlsx
+++ b/docs/migration-orders/davin-operational-manual/antigravity/migration-process-handbook-antigravity-v12.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SaaS Project\trading-alerts-saas-public\docs\migration-orders\davin-operational-manual\antigravity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4C509DE-C536-4082-99A3-6FC3A0AEBAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AF03C5E-0148-4BFE-B05C-8FB4EAF10E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7982,57 +7982,6 @@
     <xf numFmtId="0" fontId="0" fillId="26" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -8048,6 +7997,57 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11784,16 +11784,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="149" t="s">
+      <c r="A1" s="156" t="s">
         <v>2106</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
-      <c r="E1" s="130"/>
-      <c r="F1" s="130"/>
-      <c r="G1" s="130"/>
-      <c r="H1" s="130"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
+      <c r="E1" s="137"/>
+      <c r="F1" s="137"/>
+      <c r="G1" s="137"/>
+      <c r="H1" s="137"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="110" t="s">
@@ -13058,31 +13058,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="136" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
-      <c r="E1" s="130"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
+      <c r="E1" s="137"/>
     </row>
     <row r="2" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="133" t="s">
+      <c r="A2" s="145" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
+      <c r="B2" s="137"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
     </row>
     <row r="4" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="129" t="s">
+      <c r="A4" s="144" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="130"/>
-      <c r="C4" s="130"/>
-      <c r="D4" s="130"/>
-      <c r="E4" s="130"/>
+      <c r="B4" s="137"/>
+      <c r="C4" s="137"/>
+      <c r="D4" s="137"/>
+      <c r="E4" s="137"/>
     </row>
     <row r="5" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="68" t="s">
@@ -13136,13 +13136,13 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="138" t="s">
+      <c r="A9" s="143" t="s">
         <v>106</v>
       </c>
-      <c r="B9" s="130"/>
-      <c r="C9" s="130"/>
-      <c r="D9" s="130"/>
-      <c r="E9" s="130"/>
+      <c r="B9" s="137"/>
+      <c r="C9" s="137"/>
+      <c r="D9" s="137"/>
+      <c r="E9" s="137"/>
     </row>
     <row r="10" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="68" t="s">
@@ -13379,11 +13379,11 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="130"/>
-      <c r="B24" s="130"/>
-      <c r="C24" s="130"/>
-      <c r="D24" s="130"/>
-      <c r="E24" s="130"/>
+      <c r="A24" s="137"/>
+      <c r="B24" s="137"/>
+      <c r="C24" s="137"/>
+      <c r="D24" s="137"/>
+      <c r="E24" s="137"/>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="77" t="s">
@@ -13394,51 +13394,51 @@
       <c r="A26" s="68" t="s">
         <v>162</v>
       </c>
-      <c r="B26" s="137" t="s">
+      <c r="B26" s="141" t="s">
         <v>163</v>
       </c>
-      <c r="C26" s="132"/>
-      <c r="D26" s="137"/>
-      <c r="E26" s="132"/>
+      <c r="C26" s="140"/>
+      <c r="D26" s="141"/>
+      <c r="E26" s="140"/>
     </row>
     <row r="27" spans="1:5" ht="64" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="73" t="s">
         <v>164</v>
       </c>
-      <c r="B27" s="131" t="s">
+      <c r="B27" s="142" t="s">
         <v>165</v>
       </c>
-      <c r="C27" s="132"/>
-      <c r="D27" s="131" t="s">
+      <c r="C27" s="140"/>
+      <c r="D27" s="142" t="s">
         <v>166</v>
       </c>
-      <c r="E27" s="132"/>
+      <c r="E27" s="140"/>
     </row>
     <row r="28" spans="1:5" ht="64" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="73" t="s">
         <v>167</v>
       </c>
-      <c r="B28" s="131" t="s">
+      <c r="B28" s="142" t="s">
         <v>168</v>
       </c>
-      <c r="C28" s="132"/>
-      <c r="D28" s="131" t="s">
+      <c r="C28" s="140"/>
+      <c r="D28" s="142" t="s">
         <v>169</v>
       </c>
-      <c r="E28" s="132"/>
+      <c r="E28" s="140"/>
     </row>
     <row r="29" spans="1:5" ht="64" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="73" t="s">
         <v>170</v>
       </c>
-      <c r="B29" s="131" t="s">
+      <c r="B29" s="142" t="s">
         <v>171</v>
       </c>
-      <c r="C29" s="132"/>
-      <c r="D29" s="131" t="s">
+      <c r="C29" s="140"/>
+      <c r="D29" s="142" t="s">
         <v>172</v>
       </c>
-      <c r="E29" s="132"/>
+      <c r="E29" s="140"/>
     </row>
     <row r="30" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="73" t="s">
@@ -13454,11 +13454,11 @@
       <c r="E30" s="78"/>
     </row>
     <row r="31" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="130"/>
-      <c r="B31" s="130"/>
-      <c r="C31" s="130"/>
-      <c r="D31" s="130"/>
-      <c r="E31" s="130"/>
+      <c r="A31" s="137"/>
+      <c r="B31" s="137"/>
+      <c r="C31" s="137"/>
+      <c r="D31" s="137"/>
+      <c r="E31" s="137"/>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="80" t="s">
@@ -13526,13 +13526,13 @@
       <c r="E36" s="70"/>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="135" t="s">
+      <c r="A37" s="138" t="s">
         <v>192</v>
       </c>
-      <c r="B37" s="136"/>
-      <c r="C37" s="136"/>
-      <c r="D37" s="136"/>
-      <c r="E37" s="132"/>
+      <c r="B37" s="139"/>
+      <c r="C37" s="139"/>
+      <c r="D37" s="139"/>
+      <c r="E37" s="140"/>
     </row>
     <row r="38" spans="1:5" ht="230.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="79" t="s">
@@ -14322,76 +14322,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="140" t="s">
+      <c r="A1" s="151" t="s">
         <v>308</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
-      <c r="E1" s="130"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
+      <c r="E1" s="137"/>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="141" t="s">
+      <c r="A2" s="146" t="s">
         <v>309</v>
       </c>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
+      <c r="B2" s="137"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
     </row>
     <row r="4" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="143" t="s">
+      <c r="A4" s="152" t="s">
         <v>310</v>
       </c>
-      <c r="B4" s="130"/>
-      <c r="C4" s="130"/>
-      <c r="D4" s="130"/>
-      <c r="E4" s="130"/>
+      <c r="B4" s="137"/>
+      <c r="C4" s="137"/>
+      <c r="D4" s="137"/>
+      <c r="E4" s="137"/>
     </row>
     <row r="5" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="141" t="s">
+      <c r="A5" s="146" t="s">
         <v>311</v>
       </c>
-      <c r="B5" s="130"/>
-      <c r="C5" s="130"/>
-      <c r="D5" s="130"/>
-      <c r="E5" s="130"/>
+      <c r="B5" s="137"/>
+      <c r="C5" s="137"/>
+      <c r="D5" s="137"/>
+      <c r="E5" s="137"/>
     </row>
     <row r="6" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="141" t="s">
+      <c r="A6" s="146" t="s">
         <v>312</v>
       </c>
-      <c r="B6" s="130"/>
-      <c r="C6" s="130"/>
-      <c r="D6" s="130"/>
-      <c r="E6" s="130"/>
+      <c r="B6" s="137"/>
+      <c r="C6" s="137"/>
+      <c r="D6" s="137"/>
+      <c r="E6" s="137"/>
     </row>
     <row r="7" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="141" t="s">
+      <c r="A7" s="146" t="s">
         <v>313</v>
       </c>
-      <c r="B7" s="130"/>
-      <c r="C7" s="130"/>
-      <c r="D7" s="130"/>
-      <c r="E7" s="130"/>
+      <c r="B7" s="137"/>
+      <c r="C7" s="137"/>
+      <c r="D7" s="137"/>
+      <c r="E7" s="137"/>
     </row>
     <row r="8" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="141" t="s">
+      <c r="A8" s="146" t="s">
         <v>314</v>
       </c>
-      <c r="B8" s="130"/>
-      <c r="C8" s="130"/>
-      <c r="D8" s="130"/>
-      <c r="E8" s="130"/>
+      <c r="B8" s="137"/>
+      <c r="C8" s="137"/>
+      <c r="D8" s="137"/>
+      <c r="E8" s="137"/>
     </row>
     <row r="10" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="144" t="s">
+      <c r="A10" s="148" t="s">
         <v>315</v>
       </c>
-      <c r="B10" s="130"/>
-      <c r="C10" s="130"/>
-      <c r="D10" s="130"/>
-      <c r="E10" s="130"/>
+      <c r="B10" s="137"/>
+      <c r="C10" s="137"/>
+      <c r="D10" s="137"/>
+      <c r="E10" s="137"/>
     </row>
     <row r="11" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="61" t="s">
@@ -14581,11 +14581,11 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="142"/>
-      <c r="B22" s="136"/>
-      <c r="C22" s="136"/>
-      <c r="D22" s="136"/>
-      <c r="E22" s="132"/>
+      <c r="A22" s="147"/>
+      <c r="B22" s="139"/>
+      <c r="C22" s="139"/>
+      <c r="D22" s="139"/>
+      <c r="E22" s="140"/>
     </row>
     <row r="23" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="82" t="s">
@@ -14593,11 +14593,11 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="130"/>
-      <c r="B24" s="130"/>
-      <c r="C24" s="130"/>
-      <c r="D24" s="130"/>
-      <c r="E24" s="130"/>
+      <c r="A24" s="137"/>
+      <c r="B24" s="137"/>
+      <c r="C24" s="137"/>
+      <c r="D24" s="137"/>
+      <c r="E24" s="137"/>
     </row>
     <row r="25" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="59" t="s">
@@ -14639,22 +14639,22 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="145" t="s">
+      <c r="A28" s="149" t="s">
         <v>344</v>
       </c>
-      <c r="B28" s="136"/>
-      <c r="C28" s="136"/>
-      <c r="D28" s="136"/>
-      <c r="E28" s="132"/>
+      <c r="B28" s="139"/>
+      <c r="C28" s="139"/>
+      <c r="D28" s="139"/>
+      <c r="E28" s="140"/>
     </row>
     <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="141" t="s">
+      <c r="A29" s="146" t="s">
         <v>345</v>
       </c>
-      <c r="B29" s="130"/>
-      <c r="C29" s="130"/>
-      <c r="D29" s="130"/>
-      <c r="E29" s="130"/>
+      <c r="B29" s="137"/>
+      <c r="C29" s="137"/>
+      <c r="D29" s="137"/>
+      <c r="E29" s="137"/>
     </row>
     <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="82" t="s">
@@ -14662,11 +14662,11 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="130"/>
-      <c r="B31" s="130"/>
-      <c r="C31" s="130"/>
-      <c r="D31" s="130"/>
-      <c r="E31" s="130"/>
+      <c r="A31" s="137"/>
+      <c r="B31" s="137"/>
+      <c r="C31" s="137"/>
+      <c r="D31" s="137"/>
+      <c r="E31" s="137"/>
     </row>
     <row r="32" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="83" t="s">
@@ -14759,11 +14759,11 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="130"/>
-      <c r="B38" s="130"/>
-      <c r="C38" s="130"/>
-      <c r="D38" s="130"/>
-      <c r="E38" s="130"/>
+      <c r="A38" s="137"/>
+      <c r="B38" s="137"/>
+      <c r="C38" s="137"/>
+      <c r="D38" s="137"/>
+      <c r="E38" s="137"/>
     </row>
     <row r="39" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="84" t="s">
@@ -14774,67 +14774,67 @@
       <c r="A40" s="61" t="s">
         <v>366</v>
       </c>
-      <c r="B40" s="139" t="s">
+      <c r="B40" s="150" t="s">
         <v>367</v>
       </c>
-      <c r="C40" s="136"/>
-      <c r="D40" s="136"/>
-      <c r="E40" s="132"/>
+      <c r="C40" s="139"/>
+      <c r="D40" s="139"/>
+      <c r="E40" s="140"/>
     </row>
     <row r="41" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="62" t="s">
         <v>368</v>
       </c>
-      <c r="B41" s="131" t="s">
+      <c r="B41" s="142" t="s">
         <v>369</v>
       </c>
-      <c r="C41" s="136"/>
-      <c r="D41" s="136"/>
-      <c r="E41" s="132"/>
+      <c r="C41" s="139"/>
+      <c r="D41" s="139"/>
+      <c r="E41" s="140"/>
     </row>
     <row r="42" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="62" t="s">
         <v>370</v>
       </c>
-      <c r="B42" s="131" t="s">
+      <c r="B42" s="142" t="s">
         <v>371</v>
       </c>
-      <c r="C42" s="136"/>
-      <c r="D42" s="136"/>
-      <c r="E42" s="132"/>
+      <c r="C42" s="139"/>
+      <c r="D42" s="139"/>
+      <c r="E42" s="140"/>
     </row>
     <row r="43" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="62" t="s">
         <v>372</v>
       </c>
-      <c r="B43" s="131" t="s">
+      <c r="B43" s="142" t="s">
         <v>373</v>
       </c>
-      <c r="C43" s="136"/>
-      <c r="D43" s="136"/>
-      <c r="E43" s="132"/>
+      <c r="C43" s="139"/>
+      <c r="D43" s="139"/>
+      <c r="E43" s="140"/>
     </row>
     <row r="44" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="62" t="s">
         <v>374</v>
       </c>
-      <c r="B44" s="131" t="s">
+      <c r="B44" s="142" t="s">
         <v>375</v>
       </c>
-      <c r="C44" s="136"/>
-      <c r="D44" s="136"/>
-      <c r="E44" s="132"/>
+      <c r="C44" s="139"/>
+      <c r="D44" s="139"/>
+      <c r="E44" s="140"/>
     </row>
     <row r="45" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="62" t="s">
         <v>376</v>
       </c>
-      <c r="B45" s="131" t="s">
+      <c r="B45" s="142" t="s">
         <v>377</v>
       </c>
-      <c r="C45" s="136"/>
-      <c r="D45" s="136"/>
-      <c r="E45" s="132"/>
+      <c r="C45" s="139"/>
+      <c r="D45" s="139"/>
+      <c r="E45" s="140"/>
     </row>
     <row r="46" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="62" t="s">
@@ -14848,11 +14848,11 @@
       <c r="E46" s="78"/>
     </row>
     <row r="47" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="130"/>
-      <c r="B47" s="130"/>
-      <c r="C47" s="130"/>
-      <c r="D47" s="130"/>
-      <c r="E47" s="130"/>
+      <c r="A47" s="137"/>
+      <c r="B47" s="137"/>
+      <c r="C47" s="137"/>
+      <c r="D47" s="137"/>
+      <c r="E47" s="137"/>
     </row>
     <row r="48" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="83" t="s">
@@ -14927,6 +14927,14 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="A4:E4"/>
     <mergeCell ref="A47:E47"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A8:E8"/>
@@ -14940,14 +14948,6 @@
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="A4:E4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14968,20 +14968,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="153" t="s">
         <v>393</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
     </row>
     <row r="2" spans="1:4" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="141" t="s">
+      <c r="A2" s="146" t="s">
         <v>394</v>
       </c>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
+      <c r="B2" s="137"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
     </row>
     <row r="4" spans="1:4" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="52" t="s">
@@ -15040,44 +15040,44 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="147" t="s">
+      <c r="A8" s="154" t="s">
         <v>411</v>
       </c>
-      <c r="B8" s="130"/>
-      <c r="C8" s="130"/>
-      <c r="D8" s="130"/>
+      <c r="B8" s="137"/>
+      <c r="C8" s="137"/>
+      <c r="D8" s="137"/>
     </row>
     <row r="9" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="141" t="s">
+      <c r="A9" s="146" t="s">
         <v>412</v>
       </c>
-      <c r="B9" s="130"/>
-      <c r="C9" s="130"/>
-      <c r="D9" s="130"/>
+      <c r="B9" s="137"/>
+      <c r="C9" s="137"/>
+      <c r="D9" s="137"/>
     </row>
     <row r="10" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="141" t="s">
+      <c r="A10" s="146" t="s">
         <v>413</v>
       </c>
-      <c r="B10" s="130"/>
-      <c r="C10" s="130"/>
-      <c r="D10" s="130"/>
+      <c r="B10" s="137"/>
+      <c r="C10" s="137"/>
+      <c r="D10" s="137"/>
     </row>
     <row r="11" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="141" t="s">
+      <c r="A11" s="146" t="s">
         <v>414</v>
       </c>
-      <c r="B11" s="130"/>
-      <c r="C11" s="130"/>
-      <c r="D11" s="130"/>
+      <c r="B11" s="137"/>
+      <c r="C11" s="137"/>
+      <c r="D11" s="137"/>
     </row>
     <row r="13" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="147" t="s">
+      <c r="A13" s="154" t="s">
         <v>415</v>
       </c>
-      <c r="B13" s="130"/>
-      <c r="C13" s="130"/>
-      <c r="D13" s="130"/>
+      <c r="B13" s="137"/>
+      <c r="C13" s="137"/>
+      <c r="D13" s="137"/>
     </row>
     <row r="14" spans="1:4" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="52" t="s">
@@ -15164,60 +15164,60 @@
       </c>
     </row>
     <row r="21" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="147" t="s">
+      <c r="A21" s="154" t="s">
         <v>439</v>
       </c>
-      <c r="B21" s="130"/>
-      <c r="C21" s="130"/>
-      <c r="D21" s="130"/>
+      <c r="B21" s="137"/>
+      <c r="C21" s="137"/>
+      <c r="D21" s="137"/>
     </row>
     <row r="22" spans="1:4" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="133" t="s">
+      <c r="A22" s="145" t="s">
         <v>440</v>
       </c>
-      <c r="B22" s="130"/>
-      <c r="C22" s="130"/>
-      <c r="D22" s="130"/>
+      <c r="B22" s="137"/>
+      <c r="C22" s="137"/>
+      <c r="D22" s="137"/>
     </row>
     <row r="23" spans="1:4" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="133" t="s">
+      <c r="A23" s="145" t="s">
         <v>441</v>
       </c>
-      <c r="B23" s="130"/>
-      <c r="C23" s="130"/>
-      <c r="D23" s="130"/>
+      <c r="B23" s="137"/>
+      <c r="C23" s="137"/>
+      <c r="D23" s="137"/>
     </row>
     <row r="24" spans="1:4" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="133" t="s">
+      <c r="A24" s="145" t="s">
         <v>442</v>
       </c>
-      <c r="B24" s="130"/>
-      <c r="C24" s="130"/>
-      <c r="D24" s="130"/>
+      <c r="B24" s="137"/>
+      <c r="C24" s="137"/>
+      <c r="D24" s="137"/>
     </row>
     <row r="25" spans="1:4" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="133" t="s">
+      <c r="A25" s="145" t="s">
         <v>443</v>
       </c>
-      <c r="B25" s="130"/>
-      <c r="C25" s="130"/>
-      <c r="D25" s="130"/>
+      <c r="B25" s="137"/>
+      <c r="C25" s="137"/>
+      <c r="D25" s="137"/>
     </row>
     <row r="26" spans="1:4" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="133" t="s">
+      <c r="A26" s="145" t="s">
         <v>444</v>
       </c>
-      <c r="B26" s="130"/>
-      <c r="C26" s="130"/>
-      <c r="D26" s="130"/>
+      <c r="B26" s="137"/>
+      <c r="C26" s="137"/>
+      <c r="D26" s="137"/>
     </row>
     <row r="27" spans="1:4" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="133" t="s">
+      <c r="A27" s="145" t="s">
         <v>445</v>
       </c>
-      <c r="B27" s="130"/>
-      <c r="C27" s="130"/>
-      <c r="D27" s="130"/>
+      <c r="B27" s="137"/>
+      <c r="C27" s="137"/>
+      <c r="D27" s="137"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -15324,22 +15324,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="153" t="s">
         <v>462</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
-      <c r="E1" s="130"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
+      <c r="E1" s="137"/>
     </row>
     <row r="2" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="141" t="s">
+      <c r="A2" s="146" t="s">
         <v>463</v>
       </c>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
+      <c r="B2" s="137"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
     </row>
     <row r="4" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="52" t="s">
@@ -15495,13 +15495,13 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="147" t="s">
+      <c r="A14" s="154" t="s">
         <v>506</v>
       </c>
-      <c r="B14" s="130"/>
-      <c r="C14" s="130"/>
-      <c r="D14" s="130"/>
-      <c r="E14" s="130"/>
+      <c r="B14" s="137"/>
+      <c r="C14" s="137"/>
+      <c r="D14" s="137"/>
+      <c r="E14" s="137"/>
     </row>
     <row r="15" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="52" t="s">
@@ -15657,49 +15657,49 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="148" t="s">
+      <c r="A25" s="155" t="s">
         <v>548</v>
       </c>
-      <c r="B25" s="130"/>
-      <c r="C25" s="130"/>
-      <c r="D25" s="130"/>
-      <c r="E25" s="130"/>
+      <c r="B25" s="137"/>
+      <c r="C25" s="137"/>
+      <c r="D25" s="137"/>
+      <c r="E25" s="137"/>
     </row>
     <row r="26" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="141" t="s">
+      <c r="A26" s="146" t="s">
         <v>549</v>
       </c>
-      <c r="B26" s="130"/>
-      <c r="C26" s="130"/>
-      <c r="D26" s="130"/>
-      <c r="E26" s="130"/>
+      <c r="B26" s="137"/>
+      <c r="C26" s="137"/>
+      <c r="D26" s="137"/>
+      <c r="E26" s="137"/>
     </row>
     <row r="27" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="141" t="s">
+      <c r="A27" s="146" t="s">
         <v>550</v>
       </c>
-      <c r="B27" s="130"/>
-      <c r="C27" s="130"/>
-      <c r="D27" s="130"/>
-      <c r="E27" s="130"/>
+      <c r="B27" s="137"/>
+      <c r="C27" s="137"/>
+      <c r="D27" s="137"/>
+      <c r="E27" s="137"/>
     </row>
     <row r="28" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="141" t="s">
+      <c r="A28" s="146" t="s">
         <v>551</v>
       </c>
-      <c r="B28" s="130"/>
-      <c r="C28" s="130"/>
-      <c r="D28" s="130"/>
-      <c r="E28" s="130"/>
+      <c r="B28" s="137"/>
+      <c r="C28" s="137"/>
+      <c r="D28" s="137"/>
+      <c r="E28" s="137"/>
     </row>
     <row r="29" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="141" t="s">
+      <c r="A29" s="146" t="s">
         <v>552</v>
       </c>
-      <c r="B29" s="130"/>
-      <c r="C29" s="130"/>
-      <c r="D29" s="130"/>
-      <c r="E29" s="130"/>
+      <c r="B29" s="137"/>
+      <c r="C29" s="137"/>
+      <c r="D29" s="137"/>
+      <c r="E29" s="137"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -25270,105 +25270,105 @@
         <v>1424</v>
       </c>
     </row>
-    <row r="88" spans="1:18" s="156" customFormat="1" ht="166.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A88" s="150">
+    <row r="88" spans="1:18" s="33" customFormat="1" ht="166.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A88" s="29">
         <v>87</v>
       </c>
-      <c r="B88" s="151" t="s">
+      <c r="B88" s="34" t="s">
         <v>249</v>
       </c>
-      <c r="C88" s="152" t="s">
+      <c r="C88" s="35" t="s">
         <v>1144</v>
       </c>
-      <c r="D88" s="153" t="s">
+      <c r="D88" s="31" t="s">
         <v>567</v>
       </c>
-      <c r="E88" s="154"/>
-      <c r="F88" s="155" t="s">
+      <c r="E88" s="30"/>
+      <c r="F88" s="32" t="s">
         <v>1829</v>
       </c>
-      <c r="G88" s="155" t="s">
+      <c r="G88" s="32" t="s">
         <v>1830</v>
       </c>
-      <c r="H88" s="155" t="s">
+      <c r="H88" s="32" t="s">
         <v>1432</v>
       </c>
-      <c r="I88" s="155" t="s">
-        <v>1424</v>
-      </c>
-      <c r="J88" s="155" t="s">
+      <c r="I88" s="32" t="s">
+        <v>1424</v>
+      </c>
+      <c r="J88" s="32" t="s">
         <v>1433</v>
       </c>
-      <c r="K88" s="155" t="s">
+      <c r="K88" s="32" t="s">
         <v>1831</v>
       </c>
-      <c r="L88" s="153"/>
-      <c r="M88" s="153"/>
-      <c r="N88" s="155" t="s">
+      <c r="L88" s="31"/>
+      <c r="M88" s="31"/>
+      <c r="N88" s="32" t="s">
         <v>1428</v>
       </c>
-      <c r="O88" s="155" t="s">
-        <v>1424</v>
-      </c>
-      <c r="P88" s="155" t="s">
-        <v>1424</v>
-      </c>
-      <c r="Q88" s="155" t="s">
+      <c r="O88" s="32" t="s">
+        <v>1424</v>
+      </c>
+      <c r="P88" s="32" t="s">
+        <v>1424</v>
+      </c>
+      <c r="Q88" s="32" t="s">
         <v>1832</v>
       </c>
-      <c r="R88" s="155" t="s">
-        <v>1424</v>
-      </c>
-    </row>
-    <row r="89" spans="1:18" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A89" s="29">
+      <c r="R88" s="32" t="s">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="89" spans="1:18" s="135" customFormat="1" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A89" s="129">
         <v>88</v>
       </c>
-      <c r="B89" s="14" t="s">
+      <c r="B89" s="130" t="s">
         <v>1190</v>
       </c>
-      <c r="C89" s="15" t="s">
+      <c r="C89" s="131" t="s">
         <v>1191</v>
       </c>
-      <c r="D89" s="3" t="s">
+      <c r="D89" s="132" t="s">
         <v>580</v>
       </c>
-      <c r="E89" s="13" t="s">
+      <c r="E89" s="133" t="s">
         <v>1855</v>
       </c>
-      <c r="F89" s="16" t="s">
+      <c r="F89" s="134" t="s">
         <v>1856</v>
       </c>
-      <c r="G89" s="16" t="s">
+      <c r="G89" s="134" t="s">
         <v>1857</v>
       </c>
-      <c r="H89" s="16" t="s">
+      <c r="H89" s="134" t="s">
         <v>1432</v>
       </c>
-      <c r="I89" s="16"/>
-      <c r="J89" s="16" t="s">
+      <c r="I89" s="134"/>
+      <c r="J89" s="134" t="s">
         <v>1433</v>
       </c>
-      <c r="K89" s="16" t="s">
+      <c r="K89" s="134" t="s">
         <v>1858</v>
       </c>
-      <c r="L89" s="3"/>
-      <c r="M89" s="3" t="s">
+      <c r="L89" s="132"/>
+      <c r="M89" s="132" t="s">
         <v>1550</v>
       </c>
-      <c r="N89" s="16" t="s">
+      <c r="N89" s="134" t="s">
         <v>1428</v>
       </c>
-      <c r="O89" s="16" t="s">
+      <c r="O89" s="134" t="s">
         <v>1620</v>
       </c>
-      <c r="P89" s="16" t="s">
+      <c r="P89" s="134" t="s">
         <v>1859</v>
       </c>
-      <c r="Q89" s="16" t="s">
+      <c r="Q89" s="134" t="s">
         <v>1860</v>
       </c>
-      <c r="R89" s="16"/>
+      <c r="R89" s="134"/>
     </row>
     <row r="90" spans="1:18" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A90" s="29">

</xml_diff>